<commit_message>
scan: seg1 2026-06-19 01:22 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq2_2026-06-18.xlsx
+++ b/output/full_scan/batch_seq2_2026-06-18.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O148"/>
+  <dimension ref="A1:O149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5509,21 +5509,21 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>1720</v>
+        <v>1776</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>生達</t>
+          <t>展宇</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>454.4322164403017</v>
+        <v>456.2232707404281</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>62.9</v>
+        <v>18.75</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>57.55333201079053</v>
+        <v>59.02734887778634</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>14.77300939168154</v>
+        <v>20.5305565147548</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.6858228994332405</v>
+        <v>0.7846991791354222</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.0380359427277178</v>
+        <v>-0.026812845005488</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>2397</v>
+        <v>1720</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>友通</t>
+          <t>生達</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>439.0012772937849</v>
+        <v>454.4322164403017</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>60.8</v>
+        <v>62.9</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>46.49473230372926</v>
+        <v>57.55333201079053</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>24.23688713523992</v>
+        <v>14.77300939168154</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.5590615509568831</v>
+        <v>0.6858228994332405</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.468314725094468</v>
+        <v>0.0380359427277178</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>2354</v>
+        <v>2397</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>鴻準</t>
+          <t>友通</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>435.3316214944964</v>
+        <v>439.0012772937849</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>57.9</v>
+        <v>60.8</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,16 +5640,16 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>48.41562683012295</v>
+        <v>46.49473230372926</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>15.79078990167362</v>
+        <v>24.23688713523992</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.5973163706288835</v>
+        <v>0.5590615509568831</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.4800550453975925</v>
+        <v>-0.468314725094468</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>1583</v>
+        <v>2354</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>程泰</t>
+          <t>鴻準</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>433.8151345740748</v>
+        <v>435.3316214944964</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>50.3</v>
+        <v>57.9</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,16 +5693,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>47.44810123011622</v>
+        <v>48.41562683012295</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>21.24331732775949</v>
+        <v>15.79078990167362</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.2447427123961635</v>
+        <v>0.5973163706288835</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.603560360283534</v>
+        <v>-0.4800550453975925</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>2313</v>
+        <v>1583</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>華通</t>
+          <t>程泰</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>430.1782507609056</v>
+        <v>433.8151345740748</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>259.5</v>
+        <v>50.3</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,13 +5746,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>49.15914812058075</v>
+        <v>47.44810123011622</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>9.927007755344524</v>
+        <v>21.24331732775949</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.5362843606851996</v>
+        <v>0.2447427123961635</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-1.978185491606222</v>
+        <v>-0.603560360283534</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>1710</v>
+        <v>2313</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>東聯</t>
+          <t>華通</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>430.1019086822926</v>
+        <v>430.1782507609056</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>13.65</v>
+        <v>259.5</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,16 +5799,16 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>49.2737893868151</v>
+        <v>49.15914812058075</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>22.56662015430162</v>
+        <v>9.927007755344524</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.5183421252852257</v>
+        <v>0.5362843606851996</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.1270570653536874</v>
+        <v>-1.978185491606222</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>2423</v>
+        <v>1710</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>固緯</t>
+          <t>東聯</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>426.8164605853715</v>
+        <v>430.1019086822926</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>77.7</v>
+        <v>13.65</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,16 +5852,16 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>56.72079176560356</v>
+        <v>49.2737893868151</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>32.64639778385665</v>
+        <v>22.56662015430162</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.3189065302211136</v>
+        <v>0.5183421252852257</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.8631301052138824</v>
+        <v>-0.1270570653536874</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>1611</v>
+        <v>2423</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>中電</t>
+          <t>固緯</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>423.4243857452175</v>
+        <v>426.8164605853715</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>13</v>
+        <v>77.7</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,16 +5905,16 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>52.72158045310377</v>
+        <v>56.72079176560356</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>29.92230986878251</v>
+        <v>32.64639778385665</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.5331754794307815</v>
+        <v>0.3189065302211136</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.0317581253584544</v>
+        <v>-0.8631301052138824</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>1712</v>
+        <v>1611</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>興農</t>
+          <t>中電</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>423.3171453103228</v>
+        <v>423.4243857452175</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>39.3</v>
+        <v>13</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>38.31035837251645</v>
+        <v>52.72158045310377</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>39.30213837328886</v>
+        <v>29.92230986878251</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.8664510315702858</v>
+        <v>0.5331754794307815</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.1532340431290266</v>
+        <v>-0.0317581253584544</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>1595</v>
+        <v>1712</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>川寶</t>
+          <t>興農</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>422.49396679245</v>
+        <v>423.3171453103228</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>77</v>
+        <v>39.3</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,16 +6011,16 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>48.27832603173342</v>
+        <v>38.31035837251645</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>23.81193249933948</v>
+        <v>39.30213837328886</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.5090838567966948</v>
+        <v>0.8664510315702858</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-1.017339905846187</v>
+        <v>0.1532340431290266</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>2345</v>
+        <v>1595</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>智邦</t>
+          <t>川寶</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>419.5954864147937</v>
+        <v>422.49396679245</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>2435</v>
+        <v>77</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,16 +6064,16 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>50.92602519152747</v>
+        <v>48.27832603173342</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>14.56846470781617</v>
+        <v>23.81193249933948</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>1.200712957136923</v>
+        <v>0.5090838567966948</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-14.09444869488111</v>
+        <v>-1.017339905846187</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>2440</v>
+        <v>2345</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>太空梭</t>
+          <t>智邦</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>419.0077882438777</v>
+        <v>419.5954864147937</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>16.95</v>
+        <v>2435</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>46.07772982204677</v>
+        <v>50.92602519152747</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>27.54919866985365</v>
+        <v>14.56846470781617</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.2856946395114544</v>
+        <v>1.200712957136923</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.1922290203049519</v>
+        <v>-14.09444869488111</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>2331</v>
+        <v>2440</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>精英</t>
+          <t>太空梭</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>412.1607033623935</v>
+        <v>419.0077882438777</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>22.4</v>
+        <v>16.95</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,16 +6170,16 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>53.86829515555316</v>
+        <v>46.07772982204677</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>17.4553621341654</v>
+        <v>27.54919866985365</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.5596325275350118</v>
+        <v>0.2856946395114544</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.0515285077363122</v>
+        <v>-0.1922290203049519</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>1773</v>
+        <v>2331</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>勝一</t>
+          <t>精英</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>410.4537926496138</v>
+        <v>412.1607033623935</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>180</v>
+        <v>22.4</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,16 +6223,16 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>54.14097479792282</v>
+        <v>53.86829515555316</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>19.67741535751051</v>
+        <v>17.4553621341654</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>1.027458505712971</v>
+        <v>0.5596325275350118</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.5440795606209647</v>
+        <v>-0.0515285077363122</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, above_ichimoku_cloud</t>
+          <t>above_ema60, market_above_ma60, liquidity_ok, stronger_than_market, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>2421</v>
+        <v>1773</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>建準</t>
+          <t>勝一</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>409.3214215137621</v>
+        <v>410.4537926496138</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>145</v>
+        <v>180</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,16 +6276,16 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>43.17713450669962</v>
+        <v>54.14097479792282</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>15.03369068778271</v>
+        <v>19.67741535751051</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.3044047837275356</v>
+        <v>1.027458505712971</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-2.271446821153868</v>
+        <v>-0.5440795606209647</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>2385</v>
+        <v>2421</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>群光</t>
+          <t>建準</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>407.0756853029543</v>
+        <v>409.3214215137621</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>114</v>
+        <v>145</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>31.35310364251974</v>
+        <v>43.17713450669962</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>31.04397562530362</v>
+        <v>15.03369068778271</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>1.107568530295428</v>
+        <v>0.3044047837275356</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-3.488189360506487</v>
+        <v>-2.271446821153868</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, dealer_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>1618</v>
+        <v>2385</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>合機</t>
+          <t>群光</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>399.2721083236845</v>
+        <v>407.0756853029543</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>41.8</v>
+        <v>114</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>51.01936084884878</v>
+        <v>31.35310364251974</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>26.94350371042109</v>
+        <v>31.04397562530362</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.3272108323684468</v>
+        <v>1.107568530295428</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.1969023940600851</v>
+        <v>-3.488189360506487</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>2387</v>
+        <v>1618</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>精元</t>
+          <t>合機</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>398.2373355898505</v>
+        <v>399.2721083236845</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>39.5</v>
+        <v>41.8</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>42.460715651141</v>
+        <v>51.01936084884878</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>20.26982575364458</v>
+        <v>26.94350371042109</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.5455046704254408</v>
+        <v>0.3272108323684468</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-0.2716147898696506</v>
+        <v>-0.1969023940600851</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>1626</v>
+        <v>2387</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>艾美特-KY</t>
+          <t>精元</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>381.4282184668197</v>
+        <v>398.2373355898505</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>9.970000000000001</v>
+        <v>39.5</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,16 +6488,16 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>42.38138856777025</v>
+        <v>42.460715651141</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>18.22131916324105</v>
+        <v>20.26982575364458</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>2.421059411714873</v>
+        <v>0.5455046704254408</v>
       </c>
       <c r="K114" s="2" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="L114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0294370837833448</v>
+        <v>-0.2716147898696506</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>1711</v>
+        <v>1626</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>永光</t>
+          <t>艾美特-KY</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>377.1635337795963</v>
+        <v>381.4282184668197</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>45.3</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,16 +6541,16 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>45.38633409976226</v>
+        <v>42.38138856777025</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>10.22006082448852</v>
+        <v>18.22131916324105</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.7118045127105983</v>
+        <v>2.421059411714873</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="L115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.1919400122572614</v>
+        <v>0.0294370837833448</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, dealer_buy_3d</t>
+          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>1735</v>
+        <v>1711</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>日勝化</t>
+          <t>永光</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>375.2090461724536</v>
+        <v>377.1635337795963</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>23.15</v>
+        <v>45.3</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,16 +6594,16 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>41.9990022815353</v>
+        <v>45.38633409976226</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>19.96354617172346</v>
+        <v>10.22006082448852</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.6366488932859836</v>
+        <v>0.7118045127105983</v>
       </c>
       <c r="K116" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.1611946103579706</v>
+        <v>-0.1919400122572614</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>2444</v>
+        <v>1735</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>兆勁</t>
+          <t>日勝化</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>371.430496009057</v>
+        <v>375.2090461724536</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>13.4</v>
+        <v>23.15</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,16 +6647,16 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>53.66443898691742</v>
+        <v>41.9990022815353</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>14.57347259254319</v>
+        <v>19.96354617172346</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.7606582513234174</v>
+        <v>0.6366488932859836</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.0625531843153497</v>
+        <v>-0.1611946103579706</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>1752</v>
+        <v>2444</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>南光</t>
+          <t>兆勁</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>368.0899421750701</v>
+        <v>371.430496009057</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>32.8</v>
+        <v>13.4</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,16 +6700,16 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>44.74685116530853</v>
+        <v>53.66443898691742</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>18.85769985798773</v>
+        <v>14.57347259254319</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.9965907101142268</v>
+        <v>0.7606582513234174</v>
       </c>
       <c r="K118" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>0.07380045652876641</v>
+        <v>0.0625531843153497</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>2417</v>
+        <v>1752</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>圓剛</t>
+          <t>南光</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>357.5521260217886</v>
+        <v>368.0899421750701</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>46.1</v>
+        <v>32.8</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,16 +6753,16 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>46.30015213640131</v>
+        <v>44.74685116530853</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>16.33576786210864</v>
+        <v>18.85769985798773</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.4451630581558397</v>
+        <v>0.9965907101142268</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.4872433961643525</v>
+        <v>0.07380045652876641</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>2072</v>
+        <v>2417</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>世紀風電</t>
+          <t>圓剛</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>350.1288268637942</v>
+        <v>357.5521260217886</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>174</v>
+        <v>46.1</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>43.77536055097619</v>
+        <v>46.30015213640131</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>14.84502513356362</v>
+        <v>16.33576786210864</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.6065687812556201</v>
+        <v>0.4451630581558397</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6824,31 +6824,31 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.4216340707233443</v>
+        <v>-0.4872433961643525</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
+          <t>above_ema60, ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>2430</v>
+        <v>2072</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>燦坤</t>
+          <t>世紀風電</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>344.4332004069925</v>
+        <v>350.1288268637942</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>18.45</v>
+        <v>174</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,16 +6859,16 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>42.97696517802144</v>
+        <v>43.77536055097619</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>28.2380343593708</v>
+        <v>14.84502513356362</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.5263547080724265</v>
+        <v>0.6065687812556201</v>
       </c>
       <c r="K121" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L121" s="2" t="n">
         <v>0</v>
@@ -6877,31 +6877,31 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.0649186320359342</v>
+        <v>-0.4216340707233443</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>1587</v>
+        <v>2430</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>吉茂</t>
+          <t>燦坤</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>336.4459582483088</v>
+        <v>344.4332004069925</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>28.05</v>
+        <v>18.45</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,16 +6912,16 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>40.23715685292817</v>
+        <v>42.97696517802144</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>20.58687436328653</v>
+        <v>28.2380343593708</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.2892773817800352</v>
+        <v>0.5263547080724265</v>
       </c>
       <c r="K122" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L122" s="2" t="n">
         <v>0</v>
@@ -6930,31 +6930,31 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>0.0045593704273266</v>
+        <v>0.0649186320359342</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>2314</v>
+        <v>1587</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>台揚</t>
+          <t>吉茂</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>327.8013910091495</v>
+        <v>336.4459582483088</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>14.95</v>
+        <v>28.05</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,16 +6965,16 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>45.88614526175413</v>
+        <v>40.23715685292817</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>15.55895872780824</v>
+        <v>20.58687436328653</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.7062399116727571</v>
+        <v>0.2892773817800352</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L123" s="2" t="n">
         <v>0</v>
@@ -6983,31 +6983,31 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.0778387849805267</v>
+        <v>0.0045593704273266</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>1707</v>
+        <v>2314</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>葡萄王</t>
+          <t>台揚</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>326.3720851987862</v>
+        <v>327.8013910091495</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>99.7</v>
+        <v>14.95</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,16 +7018,16 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>32.06063645628821</v>
+        <v>45.88614526175413</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>48.22113065913423</v>
+        <v>15.55895872780824</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.6512368489815044</v>
+        <v>0.7062399116727571</v>
       </c>
       <c r="K124" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L124" s="2" t="n">
         <v>0</v>
@@ -7036,31 +7036,31 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.4018411258453245</v>
+        <v>-0.0778387849805267</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>1815</v>
+        <v>1707</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>富喬</t>
+          <t>葡萄王</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>300.1575362650258</v>
+        <v>326.3720851987862</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>98.09999999999999</v>
+        <v>99.7</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,16 +7071,16 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>45.88036245579491</v>
+        <v>32.06063645628821</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>16.09469352008011</v>
+        <v>48.22113065913423</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>0.7957287387956904</v>
+        <v>0.6512368489815044</v>
       </c>
       <c r="K125" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L125" s="2" t="n">
         <v>0</v>
@@ -7089,31 +7089,31 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.3086821833700837</v>
+        <v>0.4018411258453245</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>2419</v>
+        <v>1815</v>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>仲琦</t>
+          <t>富喬</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>296.430136300057</v>
+        <v>300.1575362650258</v>
       </c>
       <c r="E126" s="2" t="n">
-        <v>29.45</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
@@ -7124,16 +7124,16 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>45.82373799807361</v>
+        <v>45.88036245579491</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>13.7665617909241</v>
+        <v>16.09469352008011</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>0.3821999474205593</v>
+        <v>0.7957287387956904</v>
       </c>
       <c r="K126" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L126" s="2" t="n">
         <v>0</v>
@@ -7142,31 +7142,31 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.06906518627847991</v>
+        <v>-0.3086821833700837</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
-        <v>1733</v>
+        <v>2419</v>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>五鼎</t>
+          <t>仲琦</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
         <v/>
       </c>
       <c r="D127" s="2" t="n">
-        <v>295.5685183719795</v>
+        <v>296.430136300057</v>
       </c>
       <c r="E127" s="2" t="n">
-        <v>29.3</v>
+        <v>29.45</v>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
@@ -7177,16 +7177,16 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>47.75043312803395</v>
+        <v>45.82373799807361</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>18.85242351115028</v>
+        <v>13.7665617909241</v>
       </c>
       <c r="J127" s="2" t="n">
-        <v>0.4088870131317245</v>
+        <v>0.3821999474205593</v>
       </c>
       <c r="K127" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L127" s="2" t="n">
         <v>0</v>
@@ -7195,31 +7195,31 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.09318394793615289</v>
+        <v>-0.06906518627847991</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
-        <v>2329</v>
+        <v>1733</v>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>華泰</t>
+          <t>五鼎</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
         <v/>
       </c>
       <c r="D128" s="2" t="n">
-        <v>294.6415796915435</v>
+        <v>295.5685183719795</v>
       </c>
       <c r="E128" s="2" t="n">
-        <v>55.6</v>
+        <v>29.3</v>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
@@ -7230,16 +7230,16 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>49.17551411820892</v>
+        <v>47.75043312803395</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>10.49952319885315</v>
+        <v>18.85242351115028</v>
       </c>
       <c r="J128" s="2" t="n">
-        <v>1.297255337210825</v>
+        <v>0.4088870131317245</v>
       </c>
       <c r="K128" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L128" s="2" t="n">
         <v>0</v>
@@ -7248,31 +7248,31 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>-0.146209746436862</v>
+        <v>-0.09318394793615289</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
-        <v>1614</v>
+        <v>2329</v>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>三洋電</t>
+          <t>華泰</t>
         </is>
       </c>
       <c r="C129" s="2" t="n">
         <v/>
       </c>
       <c r="D129" s="2" t="n">
-        <v>290.3671545567316</v>
+        <v>294.6415796915435</v>
       </c>
       <c r="E129" s="2" t="n">
-        <v>31.9</v>
+        <v>55.6</v>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
@@ -7283,16 +7283,16 @@
         <v>0</v>
       </c>
       <c r="H129" s="2" t="n">
-        <v>50.53044996720536</v>
+        <v>49.17551411820892</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>17.66927110317452</v>
+        <v>10.49952319885315</v>
       </c>
       <c r="J129" s="2" t="n">
-        <v>0.7298042947241385</v>
+        <v>1.297255337210825</v>
       </c>
       <c r="K129" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L129" s="2" t="n">
         <v>0</v>
@@ -7301,31 +7301,31 @@
         <v>-1</v>
       </c>
       <c r="N129" s="2" t="n">
-        <v>-0.0211676199638906</v>
+        <v>-0.146209746436862</v>
       </c>
       <c r="O129" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
-        <v>1732</v>
+        <v>1614</v>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>毛寶</t>
+          <t>三洋電</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
         <v/>
       </c>
       <c r="D130" s="2" t="n">
-        <v>287.1337030332799</v>
+        <v>290.3671545567316</v>
       </c>
       <c r="E130" s="2" t="n">
-        <v>26.3</v>
+        <v>31.9</v>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
@@ -7336,16 +7336,16 @@
         <v>0</v>
       </c>
       <c r="H130" s="2" t="n">
-        <v>48.48273464944292</v>
+        <v>50.53044996720536</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>13.96924875192235</v>
+        <v>17.66927110317452</v>
       </c>
       <c r="J130" s="2" t="n">
-        <v>0.2702961280991005</v>
+        <v>0.7298042947241385</v>
       </c>
       <c r="K130" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L130" s="2" t="n">
         <v>0</v>
@@ -7354,31 +7354,31 @@
         <v>-1</v>
       </c>
       <c r="N130" s="2" t="n">
-        <v>-0.0265446134088996</v>
+        <v>-0.0211676199638906</v>
       </c>
       <c r="O130" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="n">
-        <v>1736</v>
+        <v>1732</v>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>喬山</t>
+          <t>毛寶</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
         <v/>
       </c>
       <c r="D131" s="2" t="n">
-        <v>273.8790548045606</v>
+        <v>287.1337030332799</v>
       </c>
       <c r="E131" s="2" t="n">
-        <v>119.5</v>
+        <v>26.3</v>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
@@ -7389,16 +7389,16 @@
         <v>0</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>54.62120259244998</v>
+        <v>48.48273464944292</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>12.65140570367837</v>
+        <v>13.96924875192235</v>
       </c>
       <c r="J131" s="2" t="n">
-        <v>1.1001317693702</v>
+        <v>0.2702961280991005</v>
       </c>
       <c r="K131" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L131" s="2" t="n">
         <v>0</v>
@@ -7407,31 +7407,31 @@
         <v>-1</v>
       </c>
       <c r="N131" s="2" t="n">
-        <v>0.9111630880006922</v>
+        <v>-0.0265446134088996</v>
       </c>
       <c r="O131" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n">
-        <v>2433</v>
+        <v>1736</v>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>互盛電</t>
+          <t>喬山</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
         <v/>
       </c>
       <c r="D132" s="2" t="n">
-        <v>267.9414113497994</v>
+        <v>273.8790548045606</v>
       </c>
       <c r="E132" s="2" t="n">
-        <v>44.5</v>
+        <v>119.5</v>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
@@ -7442,16 +7442,16 @@
         <v>0</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>52.64340755972051</v>
+        <v>54.62120259244998</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>14.30871231907714</v>
+        <v>12.65140570367837</v>
       </c>
       <c r="J132" s="2" t="n">
-        <v>0.347159996391737</v>
+        <v>1.1001317693702</v>
       </c>
       <c r="K132" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L132" s="2" t="n">
         <v>0</v>
@@ -7460,31 +7460,31 @@
         <v>-1</v>
       </c>
       <c r="N132" s="2" t="n">
-        <v>0.1311313089541053</v>
+        <v>0.9111630880006922</v>
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="n">
-        <v>2424</v>
+        <v>2433</v>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>隴華</t>
+          <t>互盛電</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
         <v/>
       </c>
       <c r="D133" s="2" t="n">
-        <v>264.4936385172006</v>
+        <v>267.9414113497994</v>
       </c>
       <c r="E133" s="2" t="n">
-        <v>10.6</v>
+        <v>44.5</v>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
@@ -7495,16 +7495,16 @@
         <v>0</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>31.99346474624188</v>
+        <v>52.64340755972051</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>28.0073209081328</v>
+        <v>14.30871231907714</v>
       </c>
       <c r="J133" s="2" t="n">
-        <v>0.7440846304046758</v>
+        <v>0.347159996391737</v>
       </c>
       <c r="K133" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L133" s="2" t="n">
         <v>0</v>
@@ -7513,31 +7513,31 @@
         <v>-1</v>
       </c>
       <c r="N133" s="2" t="n">
-        <v>0.1751784257880668</v>
+        <v>0.1311313089541053</v>
       </c>
       <c r="O133" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n">
-        <v>2367</v>
+        <v>2424</v>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>燿華</t>
+          <t>隴華</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
         <v/>
       </c>
       <c r="D134" s="2" t="n">
-        <v>262.6449934103713</v>
+        <v>264.4936385172006</v>
       </c>
       <c r="E134" s="2" t="n">
-        <v>61.3</v>
+        <v>10.6</v>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
@@ -7548,16 +7548,16 @@
         <v>0</v>
       </c>
       <c r="H134" s="2" t="n">
-        <v>44.53630928422818</v>
+        <v>31.99346474624188</v>
       </c>
       <c r="I134" s="2" t="n">
-        <v>11.78924000884352</v>
+        <v>28.0073209081328</v>
       </c>
       <c r="J134" s="2" t="n">
-        <v>0.4075982010336679</v>
+        <v>0.7440846304046758</v>
       </c>
       <c r="K134" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L134" s="2" t="n">
         <v>0</v>
@@ -7566,31 +7566,31 @@
         <v>-1</v>
       </c>
       <c r="N134" s="2" t="n">
-        <v>-0.3070383698666297</v>
+        <v>0.1751784257880668</v>
       </c>
       <c r="O134" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n">
-        <v>1721</v>
+        <v>2367</v>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>三晃</t>
+          <t>燿華</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
         <v/>
       </c>
       <c r="D135" s="2" t="n">
-        <v>260.8144853673599</v>
+        <v>262.6449934103713</v>
       </c>
       <c r="E135" s="2" t="n">
-        <v>23.8</v>
+        <v>61.3</v>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
@@ -7601,13 +7601,13 @@
         <v>0</v>
       </c>
       <c r="H135" s="2" t="n">
-        <v>41.3854121397502</v>
+        <v>44.53630928422818</v>
       </c>
       <c r="I135" s="2" t="n">
-        <v>24.5449650028133</v>
+        <v>11.78924000884352</v>
       </c>
       <c r="J135" s="2" t="n">
-        <v>0.6343368448447467</v>
+        <v>0.4075982010336679</v>
       </c>
       <c r="K135" s="2" t="n">
         <v>0</v>
@@ -7619,31 +7619,31 @@
         <v>-1</v>
       </c>
       <c r="N135" s="2" t="n">
-        <v>-0.4702442873727217</v>
+        <v>-0.3070383698666297</v>
       </c>
       <c r="O135" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
-        <v>1616</v>
+        <v>1721</v>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>億泰</t>
+          <t>三晃</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
         <v/>
       </c>
       <c r="D136" s="2" t="n">
-        <v>251.8833515948172</v>
+        <v>260.8144853673599</v>
       </c>
       <c r="E136" s="2" t="n">
-        <v>22.15</v>
+        <v>23.8</v>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
@@ -7654,13 +7654,13 @@
         <v>0</v>
       </c>
       <c r="H136" s="2" t="n">
-        <v>47.81552966134699</v>
+        <v>41.3854121397502</v>
       </c>
       <c r="I136" s="2" t="n">
-        <v>16.32882574501611</v>
+        <v>24.5449650028133</v>
       </c>
       <c r="J136" s="2" t="n">
-        <v>0.5755213203031366</v>
+        <v>0.6343368448447467</v>
       </c>
       <c r="K136" s="2" t="n">
         <v>0</v>
@@ -7672,31 +7672,31 @@
         <v>-1</v>
       </c>
       <c r="N136" s="2" t="n">
-        <v>-0.0155186863536401</v>
+        <v>-0.4702442873727217</v>
       </c>
       <c r="O136" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="n">
-        <v>2429</v>
+        <v>1616</v>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>銘旺科</t>
+          <t>億泰</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
         <v/>
       </c>
       <c r="D137" s="2" t="n">
-        <v>236.588011961424</v>
+        <v>251.8833515948172</v>
       </c>
       <c r="E137" s="2" t="n">
-        <v>38.55</v>
+        <v>22.15</v>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
@@ -7707,13 +7707,13 @@
         <v>0</v>
       </c>
       <c r="H137" s="2" t="n">
-        <v>34.9218637920861</v>
+        <v>47.81552966134699</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>14.82344381127159</v>
+        <v>16.32882574501611</v>
       </c>
       <c r="J137" s="2" t="n">
-        <v>0.5901123451092285</v>
+        <v>0.5755213203031366</v>
       </c>
       <c r="K137" s="2" t="n">
         <v>0</v>
@@ -7725,31 +7725,31 @@
         <v>-1</v>
       </c>
       <c r="N137" s="2" t="n">
-        <v>-0.5028485217136929</v>
+        <v>-0.0155186863536401</v>
       </c>
       <c r="O137" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n">
-        <v>2427</v>
+        <v>2429</v>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>三商電</t>
+          <t>銘旺科</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
         <v/>
       </c>
       <c r="D138" s="2" t="n">
-        <v>224.4620433541344</v>
+        <v>236.588011961424</v>
       </c>
       <c r="E138" s="2" t="n">
-        <v>22.3</v>
+        <v>38.55</v>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
@@ -7760,13 +7760,13 @@
         <v>0</v>
       </c>
       <c r="H138" s="2" t="n">
-        <v>50.70530402997503</v>
+        <v>34.9218637920861</v>
       </c>
       <c r="I138" s="2" t="n">
-        <v>23.60009958143364</v>
+        <v>14.82344381127159</v>
       </c>
       <c r="J138" s="2" t="n">
-        <v>0.3722714774301067</v>
+        <v>0.5901123451092285</v>
       </c>
       <c r="K138" s="2" t="n">
         <v>0</v>
@@ -7778,31 +7778,31 @@
         <v>-1</v>
       </c>
       <c r="N138" s="2" t="n">
-        <v>-0.0363070961739965</v>
+        <v>-0.5028485217136929</v>
       </c>
       <c r="O138" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="n">
-        <v>2438</v>
+        <v>2427</v>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>翔耀</t>
+          <t>三商電</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
         <v/>
       </c>
       <c r="D139" s="2" t="n">
-        <v>213.1421699851261</v>
+        <v>224.4620433541344</v>
       </c>
       <c r="E139" s="2" t="n">
-        <v>22.5</v>
+        <v>22.3</v>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
@@ -7813,13 +7813,13 @@
         <v>0</v>
       </c>
       <c r="H139" s="2" t="n">
-        <v>45.81281184302722</v>
+        <v>50.70530402997503</v>
       </c>
       <c r="I139" s="2" t="n">
-        <v>18.92068095135482</v>
+        <v>23.60009958143364</v>
       </c>
       <c r="J139" s="2" t="n">
-        <v>0.3463381180260699</v>
+        <v>0.3722714774301067</v>
       </c>
       <c r="K139" s="2" t="n">
         <v>0</v>
@@ -7831,31 +7831,31 @@
         <v>-1</v>
       </c>
       <c r="N139" s="2" t="n">
-        <v>-0.3541547009411021</v>
+        <v>-0.0363070961739965</v>
       </c>
       <c r="O139" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n">
-        <v>1760</v>
+        <v>2438</v>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>寶齡富錦</t>
+          <t>翔耀</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
         <v/>
       </c>
       <c r="D140" s="2" t="n">
-        <v>211.9473749606685</v>
+        <v>213.1421699851261</v>
       </c>
       <c r="E140" s="2" t="n">
-        <v>59.9</v>
+        <v>22.5</v>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
@@ -7866,13 +7866,13 @@
         <v>0</v>
       </c>
       <c r="H140" s="2" t="n">
-        <v>41.4849538720278</v>
+        <v>45.81281184302722</v>
       </c>
       <c r="I140" s="2" t="n">
-        <v>8.21578776256297</v>
+        <v>18.92068095135482</v>
       </c>
       <c r="J140" s="2" t="n">
-        <v>1.436134327162848</v>
+        <v>0.3463381180260699</v>
       </c>
       <c r="K140" s="2" t="n">
         <v>0</v>
@@ -7884,31 +7884,31 @@
         <v>-1</v>
       </c>
       <c r="N140" s="2" t="n">
-        <v>0.0199931198367309</v>
+        <v>-0.3541547009411021</v>
       </c>
       <c r="O140" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n">
-        <v>2321</v>
+        <v>1760</v>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>東訊</t>
+          <t>寶齡富錦</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
         <v/>
       </c>
       <c r="D141" s="2" t="n">
-        <v>211.45554510959</v>
+        <v>211.9473749606685</v>
       </c>
       <c r="E141" s="2" t="n">
-        <v>14.05</v>
+        <v>59.9</v>
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
@@ -7919,13 +7919,13 @@
         <v>0</v>
       </c>
       <c r="H141" s="2" t="n">
-        <v>53.85354988137411</v>
+        <v>41.4849538720278</v>
       </c>
       <c r="I141" s="2" t="n">
-        <v>9.089294522988627</v>
+        <v>8.21578776256297</v>
       </c>
       <c r="J141" s="2" t="n">
-        <v>0.8207416231646261</v>
+        <v>1.436134327162848</v>
       </c>
       <c r="K141" s="2" t="n">
         <v>0</v>
@@ -7937,31 +7937,31 @@
         <v>-1</v>
       </c>
       <c r="N141" s="2" t="n">
-        <v>0.2734942019269837</v>
+        <v>0.0199931198367309</v>
       </c>
       <c r="O141" s="2" t="inlineStr">
         <is>
-          <t>above_ema60, market_above_ma60, obv_uptrend, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n">
-        <v>2365</v>
+        <v>2321</v>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>昆盈</t>
+          <t>東訊</t>
         </is>
       </c>
       <c r="C142" s="2" t="n">
         <v/>
       </c>
       <c r="D142" s="2" t="n">
-        <v>211.1187416165806</v>
+        <v>211.45554510959</v>
       </c>
       <c r="E142" s="2" t="n">
-        <v>34.05</v>
+        <v>14.05</v>
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
@@ -7972,16 +7972,16 @@
         <v>0</v>
       </c>
       <c r="H142" s="2" t="n">
-        <v>44.13161907077893</v>
+        <v>53.85354988137411</v>
       </c>
       <c r="I142" s="2" t="n">
-        <v>17.72167215172423</v>
+        <v>9.089294522988627</v>
       </c>
       <c r="J142" s="2" t="n">
-        <v>0.3985408554298814</v>
+        <v>0.8207416231646261</v>
       </c>
       <c r="K142" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L142" s="2" t="n">
         <v>0</v>
@@ -7990,31 +7990,31 @@
         <v>-1</v>
       </c>
       <c r="N142" s="2" t="n">
-        <v>-0.3327681630347754</v>
+        <v>0.2734942019269837</v>
       </c>
       <c r="O142" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>above_ema60, market_above_ma60, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n">
-        <v>1598</v>
+        <v>2365</v>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>岱宇</t>
+          <t>昆盈</t>
         </is>
       </c>
       <c r="C143" s="2" t="n">
         <v/>
       </c>
       <c r="D143" s="2" t="n">
-        <v>205.1087547382721</v>
+        <v>211.1187416165806</v>
       </c>
       <c r="E143" s="2" t="n">
-        <v>20.2</v>
+        <v>34.05</v>
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
@@ -8025,16 +8025,16 @@
         <v>0</v>
       </c>
       <c r="H143" s="2" t="n">
-        <v>43.09137072323583</v>
+        <v>44.13161907077893</v>
       </c>
       <c r="I143" s="2" t="n">
-        <v>10.25462798072918</v>
+        <v>17.72167215172423</v>
       </c>
       <c r="J143" s="2" t="n">
-        <v>0.8097156090038344</v>
+        <v>0.3985408554298814</v>
       </c>
       <c r="K143" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L143" s="2" t="n">
         <v>0</v>
@@ -8043,31 +8043,31 @@
         <v>-1</v>
       </c>
       <c r="N143" s="2" t="n">
-        <v>-0.0663399466337075</v>
+        <v>-0.3327681630347754</v>
       </c>
       <c r="O143" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n">
-        <v>2374</v>
+        <v>1598</v>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>佳能</t>
+          <t>岱宇</t>
         </is>
       </c>
       <c r="C144" s="2" t="n">
         <v/>
       </c>
       <c r="D144" s="2" t="n">
-        <v>197.1854038680517</v>
+        <v>205.1087547382721</v>
       </c>
       <c r="E144" s="2" t="n">
-        <v>75.3</v>
+        <v>20.2</v>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
@@ -8078,13 +8078,13 @@
         <v>0</v>
       </c>
       <c r="H144" s="2" t="n">
-        <v>46.19045604771931</v>
+        <v>43.09137072323583</v>
       </c>
       <c r="I144" s="2" t="n">
-        <v>13.36743195596134</v>
+        <v>10.25462798072918</v>
       </c>
       <c r="J144" s="2" t="n">
-        <v>0.4139893320553073</v>
+        <v>0.8097156090038344</v>
       </c>
       <c r="K144" s="2" t="n">
         <v>0</v>
@@ -8096,31 +8096,31 @@
         <v>-1</v>
       </c>
       <c r="N144" s="2" t="n">
-        <v>-0.4744570800046346</v>
+        <v>-0.0663399466337075</v>
       </c>
       <c r="O144" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="n">
-        <v>1717</v>
+        <v>2374</v>
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>長興</t>
+          <t>佳能</t>
         </is>
       </c>
       <c r="C145" s="2" t="n">
         <v/>
       </c>
       <c r="D145" s="2" t="n">
-        <v>194.135658520802</v>
+        <v>197.1854038680517</v>
       </c>
       <c r="E145" s="2" t="n">
-        <v>72.40000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
@@ -8131,25 +8131,25 @@
         <v>0</v>
       </c>
       <c r="H145" s="2" t="n">
-        <v>45.28126863287528</v>
+        <v>46.19045604771931</v>
       </c>
       <c r="I145" s="2" t="n">
-        <v>18.16737514483994</v>
+        <v>13.36743195596134</v>
       </c>
       <c r="J145" s="2" t="n">
-        <v>0.4168128496718876</v>
+        <v>0.4139893320553073</v>
       </c>
       <c r="K145" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L145" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M145" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N145" s="2" t="n">
-        <v>-0.5802429690255213</v>
+        <v>-0.4744570800046346</v>
       </c>
       <c r="O145" s="2" t="inlineStr">
         <is>
@@ -8159,21 +8159,21 @@
     </row>
     <row r="146">
       <c r="A146" s="2" t="n">
-        <v>1603</v>
+        <v>1717</v>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>華電</t>
+          <t>長興</t>
         </is>
       </c>
       <c r="C146" s="2" t="n">
         <v/>
       </c>
       <c r="D146" s="2" t="n">
-        <v>160.3505592543951</v>
+        <v>194.135658520802</v>
       </c>
       <c r="E146" s="2" t="n">
-        <v>31.7</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
@@ -8184,49 +8184,49 @@
         <v>0</v>
       </c>
       <c r="H146" s="2" t="n">
-        <v>48.678204800381</v>
+        <v>45.28126863287528</v>
       </c>
       <c r="I146" s="2" t="n">
-        <v>13.79326352279893</v>
+        <v>18.16737514483994</v>
       </c>
       <c r="J146" s="2" t="n">
-        <v>0.5962183572359744</v>
+        <v>0.4168128496718876</v>
       </c>
       <c r="K146" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L146" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M146" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N146" s="2" t="n">
-        <v>-0.0162768628797365</v>
+        <v>-0.5802429690255213</v>
       </c>
       <c r="O146" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n">
-        <v>1604</v>
+        <v>1603</v>
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>聲寶</t>
+          <t>華電</t>
         </is>
       </c>
       <c r="C147" s="2" t="n">
         <v/>
       </c>
       <c r="D147" s="2" t="n">
-        <v>107.8247907453208</v>
+        <v>160.3505592543951</v>
       </c>
       <c r="E147" s="2" t="n">
-        <v>23.15</v>
+        <v>31.7</v>
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
@@ -8237,13 +8237,13 @@
         <v>0</v>
       </c>
       <c r="H147" s="2" t="n">
-        <v>43.95865490169494</v>
+        <v>48.678204800381</v>
       </c>
       <c r="I147" s="2" t="n">
-        <v>14.9872764524067</v>
+        <v>13.79326352279893</v>
       </c>
       <c r="J147" s="2" t="n">
-        <v>0.8982528493563364</v>
+        <v>0.5962183572359744</v>
       </c>
       <c r="K147" s="2" t="n">
         <v>0</v>
@@ -8255,62 +8255,115 @@
         <v>-1</v>
       </c>
       <c r="N147" s="2" t="n">
-        <v>-0.0061918141603981</v>
+        <v>-0.0162768628797365</v>
       </c>
       <c r="O147" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n">
+        <v>1604</v>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>聲寶</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D148" s="2" t="n">
+        <v>107.8247907453208</v>
+      </c>
+      <c r="E148" s="2" t="n">
+        <v>23.15</v>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H148" s="2" t="n">
+        <v>43.95865490169494</v>
+      </c>
+      <c r="I148" s="2" t="n">
+        <v>14.9872764524067</v>
+      </c>
+      <c r="J148" s="2" t="n">
+        <v>0.8982528493563364</v>
+      </c>
+      <c r="K148" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L148" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M148" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N148" s="2" t="n">
+        <v>-0.0061918141603981</v>
+      </c>
+      <c r="O148" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="n">
         <v>1623</v>
       </c>
-      <c r="B148" s="2" t="inlineStr">
+      <c r="B149" s="2" t="inlineStr">
         <is>
           <t>大東電</t>
         </is>
       </c>
-      <c r="C148" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D148" s="2" t="n">
+      <c r="C149" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D149" s="2" t="n">
         <v>73.64508708761733</v>
       </c>
-      <c r="E148" s="2" t="n">
+      <c r="E149" s="2" t="n">
         <v>220</v>
       </c>
-      <c r="F148" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="G148" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H148" s="2" t="n">
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H149" s="2" t="n">
         <v>47.25507423899008</v>
       </c>
-      <c r="I148" s="2" t="n">
+      <c r="I149" s="2" t="n">
         <v>19.1444111177983</v>
       </c>
-      <c r="J148" s="2" t="n">
+      <c r="J149" s="2" t="n">
         <v>0.5152268171931759</v>
       </c>
-      <c r="K148" s="2" t="n">
+      <c r="K149" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="L148" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M148" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N148" s="2" t="n">
+      <c r="L149" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M149" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N149" s="2" t="n">
         <v>-1.720384156239099</v>
       </c>
-      <c r="O148" s="2" t="inlineStr">
+      <c r="O149" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, liquidity_ok</t>
         </is>

</xml_diff>